<commit_message>
Kits planos EN: remontaje tras la ronda de revisión y republicación en dl/ (VPS)
seafood, bakery, food truck: montaje idempotente, gates VERDE 8/0 (G5 y G6 N/A), autotest 16/16 · 16/16 · 14/14,
censo-entregables 0, no-latinos 0, LIT255 verde; censo, pendientes y volcados EN regenerados.

Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bakery-checklist-templates/01-bakery-opening-closing-checklist.xlsx
+++ b/astro-site/public/dl/bakery-checklist-templates/01-bakery-opening-closing-checklist.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Turn on the ovens: proofer, deck / rack oven</t>
+          <t>Turn on the ovens and the proofer: deck / rack oven</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>3:00 AM</t>
+          <t>3:30 AM</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr"/>
@@ -1204,25 +1204,25 @@
       <c r="E28" s="6" t="inlineStr"/>
       <c r="F28" s="6" t="inlineStr"/>
     </row>
-    <row r="29" ht="74" customHeight="1">
+    <row r="29" ht="33.25" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Check ovens are off and clean; gas ovens: burners, gaskets and connections serviced by a licensed technician as your local code requires. Gas smell: light nothing, get out and call the gas company or 911 from outside</t>
+          <t>Count day-old bread: donate, make breadcrumbs or croutons</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Baker</t>
+          <t>Counter staff</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>2:30 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr"/>
@@ -1231,17 +1231,17 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>General</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Count day-old bread: donate, make breadcrumbs or croutons</t>
+          <t>Order flour and ingredients for tomorrow</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Counter staff</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -1252,20 +1252,20 @@
       <c r="E30" s="6" t="inlineStr"/>
       <c r="F30" s="6" t="inlineStr"/>
     </row>
-    <row r="31" ht="33.25" customHeight="1">
+    <row r="31" ht="74" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Shop</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Close out the register and log sales: cash count and over/short against the POS Z report</t>
+          <t>Check ovens are off and clean; gas ovens: burners, gaskets and connections serviced by a licensed technician as your local code requires. Gas smell: light nothing, get out and call the gas company or 911 from outside</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Baker</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -1276,15 +1276,15 @@
       <c r="E31" s="6" t="inlineStr"/>
       <c r="F31" s="6" t="inlineStr"/>
     </row>
-    <row r="32" ht="20" customHeight="1">
+    <row r="32" ht="33.25" customHeight="1">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Order flour and ingredients for tomorrow</t>
+          <t>Close out the register and log sales: cash count and over/short against the POS Z report</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>2:30 PM</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr"/>

</xml_diff>